<commit_message>
feat: enhance WebSocket stability, JSON serialization, and suggestion endpoints with updated timeouts
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2423,13 +2423,11 @@
           <t>show 5 schools in guntur</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>Empty query</t>
@@ -2443,6 +2441,329 @@
       </c>
       <c r="K50" t="n">
         <v>52.64</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-22 22:29:15</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>sess_18979e</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-22 22:37:02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>sess_1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Show students</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SELECT * FROM dim_student</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-22 22:49:37</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>sess_d985b1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-22 22:49:44</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>sess_date_test</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Show students with dob and gpa</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SELECT student_id, dob, gpa FROM dim_student</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-22 22:50:18</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>prakhar</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>sess_real_test_1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>How many male and female citizens are in the BC social category?</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SELECT gender, COUNT(person_id) as citizen_count FROM dim_person WHERE social_category = 'BC' GROUP BY gender;</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>The query ran successfully but returned no data.</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="K55" t="n">
+        <v>16.06</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-22 23:35:54</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>session_1790100314459_pc3mw</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>How many male and female citizens are in the BC social category?</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SELECT gender, COUNT(person_id) as citizen_count FROM dim_person WHERE social_category = 'BC' GROUP BY gender;</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>The query ran successfully but returned no data.</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="K56" t="n">
+        <v>3.18</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-22 23:42:51</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>sess_6ff5e6</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add vLLM backend support for LLM chat and embeddings
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2755,7 +2755,6 @@
           <t>Here is the query result.</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="n">
         <v>0.05</v>
       </c>
@@ -2763,6 +2762,99 @@
         <v>0.02</v>
       </c>
       <c r="K57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-24 08:46:59</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>sess_028605</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-24 08:54:08</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>sess_33ac39</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K59" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: decouple embedding provider from chat backend with new EMBEDDING_PROVIDER configuration and health checks
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2847,7 +2847,6 @@
           <t>Here is the query result.</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="n">
         <v>0.05</v>
       </c>
@@ -2855,6 +2854,53 @@
         <v>0.02</v>
       </c>
       <c r="K59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-25 21:28:16</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>sess_d08299</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K60" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add reasoning configuration to disable model thinking tags
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2893,7 +2893,6 @@
           <t>Here is the query result.</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="n">
         <v>0.05</v>
       </c>
@@ -2901,6 +2900,53 @@
         <v>0.02</v>
       </c>
       <c r="K60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-25 21:37:38</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>sess_d07631</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K61" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add TOTP-authenticated live log streaming, endpoints, and comprehensive tests
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2939,7 +2939,6 @@
           <t>Here is the query result.</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="n">
         <v>0.05</v>
       </c>
@@ -2947,6 +2946,53 @@
         <v>0.02</v>
       </c>
       <c r="K61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-25 21:51:21</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>sess_b20eb5</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K62" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add content guardrails for input validation and safety checking
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2985,7 +2985,6 @@
           <t>Here is the query result.</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="n">
         <v>0.05</v>
       </c>
@@ -2993,6 +2992,467 @@
         <v>0.02</v>
       </c>
       <c r="K62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:24:20</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>sess_adb5f3</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:24:45</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>sess_e77bba</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:24:45</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>87dfa5a8-3db0-46f0-bfa1-3dfba38be7e6</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>asdfghjklqwerty</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>I cannot process this query. Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Content Policy Violation: Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:26:25</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>f2c7f144-f9fc-4ce9-824b-ef87733f2166</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>asdfghjklqwerty</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>I cannot process this query. Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Content Policy Violation: Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:26:39</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>sess_0cf32c</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:26:39</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>bad942ed-ae2f-42a8-b1bb-c0e3da90a2fb</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>asdfghjklqwerty</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>I cannot process this query. Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Content Policy Violation: Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:38:04</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>sess_ec39aa</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:38:04</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>d42d37ef-dc9d-47dc-bc09-898d73d24fff</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>asdfghjklqwerty</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>I cannot process this query. Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Content Policy Violation: Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:45:01</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>sess_48fd4d</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>What are dropouts in Guntur?</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>SELECT district, COUNT(*) FROM dropouts GROUP BY district</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-25 22:45:01</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>9b822578-4842-4779-afe1-d8e8829fb366</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>asdfghjklqwerty</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>I cannot process this query. Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Content Policy Violation: Query appears to be gibberish or nonsensical input.</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add APM and trace highlight badges to logs UI and update logging configuration
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3430,7 +3430,6 @@
           <t>asdfghjklqwerty</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>blocked</t>
@@ -3453,6 +3452,99 @@
         <v>0</v>
       </c>
       <c r="K72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-28 21:52:45</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ws_tester_563fe7</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>sess_9709a4a5</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>How many students are there?</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) FROM students;</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-28 21:52:45</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ws_tester_563fe7</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>sess_9709a4a5</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Now filter by female students</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) FROM students;</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Here is the query result.</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K74" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>